<commit_message>
Added citations using zotero, transformd table on the index.qmd to a summary table, shortened npd (to use as a model) for others
</commit_message>
<xml_diff>
--- a/administrative-database-guidance/data/tbl_npd_variables.xlsx
+++ b/administrative-database-guidance/data/tbl_npd_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Documents\technicalguide\administrative-database-guidance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B46135-951E-4A59-9EC1-52E01F27BA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984C46C6-4733-438C-959C-DA29271AD5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6015" yWindow="345" windowWidth="21090" windowHeight="14715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60840" yWindow="8235" windowWidth="21240" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,35 +25,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="26">
-  <si>
-    <t>Children who attended school in England</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
   <si>
     <t>School census (2001/02 to 2025/26)</t>
   </si>
   <si>
-    <t>Absences and exclusions (2005/06 to 2024/25)</t>
-  </si>
-  <si>
     <t>Children looked after (2005/06 to 2024/25)</t>
   </si>
   <si>
     <t>Individual-level and school level (not class level).</t>
   </si>
   <si>
-    <t>Managed by the Department for Education (DfE). Access is highly restricted and requires submitting an application through the DfE Data Sharing Service. Approved data is made available via the ONS Secure Research Service (SRS), so researchers must hold ONS Accredited Researcher status to access it.</t>
-  </si>
-  <si>
-    <t>EYFSP, KS1 and KS2 attainment data are missing for pupils who attended independent or non-state schools, as these schools do not submit statutory assessment returns.</t>
-  </si>
-  <si>
-    <t>The NPD school census includes only state-funded pupils. Independent schools do not provide pupil-level characteristics, even though they complete an annual census.</t>
-  </si>
-  <si>
-    <t>Population covered</t>
-  </si>
-  <si>
     <t>Key variables</t>
   </si>
   <si>
@@ -63,18 +45,7 @@
     <t>Unit of observation</t>
   </si>
   <si>
-    <t>Major limitations</t>
-  </si>
-  <si>
-    <t>Access and governance</t>
-  </si>
-  <si>
     <t xml:space="preserve">Child level variables such as gender, date of birth, ethnicity, postcode language, free school meal eligibility, special educational needs, social care status (looked after children and children in need), absences, exclusion, dates of joining and leaving a school. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Achievement level variables such as attainment at Key Stage 1, 2, 3, 4 and 5 (KS1, KS2, KS3, KS4 and KS5), and information about what they did after they finished school. 
-Area-based variables such as the local authority area in which the child lives.  </t>
   </si>
   <si>
     <t>School-level variables such as the local authority of the school and the school name.</t>
@@ -99,13 +70,26 @@
 Children in Need (2008/09 to 2024/25)</t>
   </si>
   <si>
-    <t>Exclusions data captured from 2001/02 to 2004/05 at school level. From 2005/06 it is at an individual level.</t>
-  </si>
-  <si>
-    <t>NPD school-level datasets provide aggregated attainment and census indicators at the level of the school (one row per school). School-level datasets summarise outcomes such as KS2–KS5 performance, contextual characteristics, and accountability measures at the individual level.</t>
-  </si>
-  <si>
     <t>Area-based variables such as the local authority area in which the child lives. </t>
+  </si>
+  <si>
+    <t>Population covered</t>
+  </si>
+  <si>
+    <t>Pupils in state-funded nursery, primary, secondary, and special schools, non-maintained special schools, pupil referral units, general hospital schools, and independent schools.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Achievement level variables such as attainment at Key Stage 1, 2, 3, 4 and 5 (KS1, KS2, KS3, KS4 and KS5), and information about what they did after they finished school. </t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Information</t>
+  </si>
+  <si>
+    <t>Absences (2005/06 to 2024/25) and exclusions (2001/2 to 2004/5 at the school level; 2005/06 to 2024/25 at an individual level)</t>
   </si>
 </sst>
 </file>
@@ -426,172 +410,143 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="71.140625" customWidth="1"/>
+    <col min="1" max="1" width="26.7265625" customWidth="1"/>
+    <col min="2" max="2" width="71.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="59" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="69.75" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>5</v>
-      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.75">
+      <c r="B19" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>